<commit_message>
Update planning: add boost tests, payment account, English, pack publishing
</commit_message>
<xml_diff>
--- a/Planning_Lancement_Kittab.xlsx
+++ b/Planning_Lancement_Kittab.xlsx
@@ -165,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -235,6 +235,15 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -601,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2208,68 +2217,242 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="28" customHeight="1">
-      <c r="A55" s="21" t="inlineStr">
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="24" t="inlineStr">
+        <is>
+          <t>Semaine 1</t>
+        </is>
+      </c>
+      <c r="B54" s="24" t="inlineStr">
+        <is>
+          <t>22-28 juin</t>
+        </is>
+      </c>
+      <c r="C54" s="24" t="inlineStr">
+        <is>
+          <t>🔧 Technique</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Tester la publication d'un pack de livres (formulaire + affichage)</t>
+        </is>
+      </c>
+      <c r="E54" s="24" t="inlineStr">
+        <is>
+          <t>🔴 Haute</t>
+        </is>
+      </c>
+      <c r="F54" s="24" t="inlineStr">
+        <is>
+          <t>☐ À faire</t>
+        </is>
+      </c>
+      <c r="G54" s="24" t="inlineStr"/>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="25" t="inlineStr">
+        <is>
+          <t>Semaine 1</t>
+        </is>
+      </c>
+      <c r="B55" s="25" t="inlineStr">
+        <is>
+          <t>22-28 juin</t>
+        </is>
+      </c>
+      <c r="C55" s="25" t="inlineStr">
+        <is>
+          <t>🔧 Technique</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>Tester la disponibilité du site en anglais (i18n, libellés)</t>
+        </is>
+      </c>
+      <c r="E55" s="25" t="inlineStr">
+        <is>
+          <t>🟡 Moyenne</t>
+        </is>
+      </c>
+      <c r="F55" s="25" t="inlineStr">
+        <is>
+          <t>☐ À faire</t>
+        </is>
+      </c>
+      <c r="G55" s="25" t="inlineStr"/>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="26" t="inlineStr">
+        <is>
+          <t>Semaine 2</t>
+        </is>
+      </c>
+      <c r="B56" s="26" t="inlineStr">
+        <is>
+          <t>29 juin - 5 juil</t>
+        </is>
+      </c>
+      <c r="C56" s="26" t="inlineStr">
+        <is>
+          <t>🔧 Technique</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>Tester le système de boost (création, affichage, expiration)</t>
+        </is>
+      </c>
+      <c r="E56" s="26" t="inlineStr">
+        <is>
+          <t>🔴 Haute</t>
+        </is>
+      </c>
+      <c r="F56" s="26" t="inlineStr">
+        <is>
+          <t>☐ À faire</t>
+        </is>
+      </c>
+      <c r="G56" s="26" t="inlineStr">
+        <is>
+          <t>⚠️ Vérifier priorité d'affichage</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="25" t="inlineStr">
+        <is>
+          <t>Semaine 2</t>
+        </is>
+      </c>
+      <c r="B57" s="25" t="inlineStr">
+        <is>
+          <t>29 juin - 5 juil</t>
+        </is>
+      </c>
+      <c r="C57" s="25" t="inlineStr">
+        <is>
+          <t>💰 Paiement</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>Créer/configurer le compte de réception des paiements boosts (Wave, Orange Money, Stripe...)</t>
+        </is>
+      </c>
+      <c r="E57" s="25" t="inlineStr">
+        <is>
+          <t>🔴 Critique</t>
+        </is>
+      </c>
+      <c r="F57" s="25" t="inlineStr">
+        <is>
+          <t>☐ À faire</t>
+        </is>
+      </c>
+      <c r="G57" s="25" t="inlineStr">
+        <is>
+          <t>⚠️ Obligatoire avant lancement</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="26" t="inlineStr">
+        <is>
+          <t>Semaine 2</t>
+        </is>
+      </c>
+      <c r="B58" s="26" t="inlineStr">
+        <is>
+          <t>29 juin - 5 juil</t>
+        </is>
+      </c>
+      <c r="C58" s="26" t="inlineStr">
+        <is>
+          <t>💰 Paiement</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>Intégrer ou simuler le flux de paiement boost (lien paiement → activation)</t>
+        </is>
+      </c>
+      <c r="E58" s="26" t="inlineStr">
+        <is>
+          <t>🔴 Haute</t>
+        </is>
+      </c>
+      <c r="F58" s="26" t="inlineStr">
+        <is>
+          <t>☐ À faire</t>
+        </is>
+      </c>
+      <c r="G58" s="26" t="inlineStr"/>
+    </row>
+    <row r="59" ht="18" customHeight="1"/>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="21" t="inlineStr">
         <is>
           <t>📊 OBJECTIFS J+7 APRÈS LANCEMENT</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="3" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
         <is>
           <t>Métrique</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>Objectif J+7</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="22" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="22" t="inlineStr">
         <is>
           <t>Inscriptions</t>
         </is>
       </c>
-      <c r="B57" s="23" t="inlineStr">
+      <c r="B62" s="23" t="inlineStr">
         <is>
           <t>100+</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="22" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="22" t="inlineStr">
         <is>
           <t>Annonces publiées</t>
         </is>
       </c>
-      <c r="B58" s="23" t="inlineStr">
+      <c r="B63" s="23" t="inlineStr">
         <is>
           <t>30+</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="22" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="22" t="inlineStr">
         <is>
           <t>Messages envoyés</t>
         </is>
       </c>
-      <c r="B59" s="23" t="inlineStr">
+      <c r="B64" s="23" t="inlineStr">
         <is>
           <t>50+</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="22" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="22" t="inlineStr">
         <is>
           <t>Villes représentées</t>
         </is>
       </c>
-      <c r="B60" s="23" t="inlineStr">
+      <c r="B65" s="23" t="inlineStr">
         <is>
           <t>3+</t>
         </is>

</xml_diff>